<commit_message>
Add data model generator, SQL Server schema, ER diagrams, local inspection database and VS Code setup
- tools/data_model: rebuilds the workbook, remap, data dictionary, SQL schema and diagrams (build_all.py)
- schema_sqlserver.sql: 57 tables, 385 foreign keys, descriptions as extended properties
- ID types made consistent so every link is a real foreign key (small lookup tables use INT keys)
- docker-compose.db.yml and db_up.py: local SQL Server with the schema loaded (schema only)
- .vscode: interpreter, tests, database connection profile, tasks, recommended extensions
- docs/ARCHITECTURE.md: the ecosystem, the 15 agents, data flow and how to inspect it
- ruff excludes tools/data_model

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_model/KrisnnAI-Canonical-Data-Model.xlsx
+++ b/docs/data_model/KrisnnAI-Canonical-Data-Model.xlsx
@@ -4754,7 +4754,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -9870,7 +9870,7 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D152" s="5" t="inlineStr">
@@ -15274,7 +15274,7 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D296" s="5" t="inlineStr">
@@ -16654,7 +16654,7 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D333" s="5" t="inlineStr">
@@ -47298,7 +47298,7 @@
       </c>
       <c r="C1154" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1154" s="6" t="inlineStr">
@@ -47770,7 +47770,7 @@
       </c>
       <c r="C1167" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1167" s="6" t="inlineStr">
@@ -48394,7 +48394,7 @@
       </c>
       <c r="C1184" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1184" s="6" t="inlineStr">
@@ -49086,7 +49086,7 @@
       </c>
       <c r="C1203" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1203" s="6" t="inlineStr">
@@ -49850,7 +49850,7 @@
       </c>
       <c r="C1224" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1224" s="6" t="inlineStr">
@@ -50462,7 +50462,7 @@
       </c>
       <c r="C1241" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1241" s="6" t="inlineStr">
@@ -50930,7 +50930,7 @@
       </c>
       <c r="C1254" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1254" s="6" t="inlineStr">
@@ -51398,7 +51398,7 @@
       </c>
       <c r="C1267" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1267" s="6" t="inlineStr">
@@ -51830,7 +51830,7 @@
       </c>
       <c r="C1279" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1279" s="6" t="inlineStr">
@@ -55538,7 +55538,7 @@
       </c>
       <c r="C1379" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1379" s="6" t="inlineStr">
@@ -57126,7 +57126,7 @@
       </c>
       <c r="C1422" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1422" s="6" t="inlineStr">
@@ -57846,7 +57846,7 @@
       </c>
       <c r="C1442" s="4" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D1442" s="6" t="inlineStr">

</xml_diff>